<commit_message>
Drop Recommendation 4 (Direct Plan Migration) from the analysis workbook
Removed at the client's instruction. Recommendations 1 to 3 are unchanged
and still reproduced in full; nothing else on the sheet moves, and the
other four sheets are untouched.

The two Week 1 items in the 30-Day Action Plan still mention Direct plans
("switching to Direct plans", "Regular vs Direct") - they are separate
entries in the report's own plan, so they are left in place pending a
decision on them.

recalc reports 0 errors over 95 formulas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TGF2E3hT6nLFch7z9VKTD7
</commit_message>
<xml_diff>
--- a/Portfolio_Fund_Analysis.xlsx
+++ b/Portfolio_Fund_Analysis.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="226">
   <si>
     <t xml:space="preserve">PORTFOLIO FUND ANALYSIS REPORT</t>
   </si>
@@ -648,24 +648,6 @@
   </si>
   <si>
     <t xml:space="preserve">Phase 4 (Months 4-6): Finalize rebalancing and tax documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recommendation 4: Consider Direct Plan Migration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Switching from Regular to Direct plans can save Rs 2-3 lakh annually in fees.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review your relationship with your fund distributor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculate tax cost of switching vs. long-term fee savings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direct plans typically have 0.5-1.5% lower expense ratios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Over 10 years: Direct plans can add Rs 23+ lakh to your portfolio</t>
   </si>
   <si>
     <t xml:space="preserve">ACTION PLAN: NEXT 30 DAYS</t>
@@ -1508,11 +1490,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="24156273"/>
-        <c:axId val="36557543"/>
+        <c:axId val="63393361"/>
+        <c:axId val="57466718"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="24156273"/>
+        <c:axId val="63393361"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1544,7 +1526,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36557543"/>
+        <c:crossAx val="57466718"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1552,7 +1534,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36557543"/>
+        <c:axId val="57466718"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1594,7 +1576,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24156273"/>
+        <c:crossAx val="63393361"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3835,7 +3817,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -4026,174 +4008,120 @@
       <c r="E23" s="46"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="36" t="s">
+      <c r="A25" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="B25" s="36"/>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="44" t="s">
+      <c r="A26" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="B26" s="44"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="44"/>
-    </row>
-    <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25"/>
+      <c r="B26" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="47" t="s">
+        <v>212</v>
+      </c>
       <c r="B27" s="45" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C27" s="45"/>
       <c r="D27" s="24"/>
       <c r="E27" s="46"/>
     </row>
-    <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25"/>
+    <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="47" t="s">
+        <v>212</v>
+      </c>
       <c r="B28" s="45" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C28" s="45"/>
       <c r="D28" s="24"/>
       <c r="E28" s="46"/>
     </row>
-    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="25"/>
+    <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="47" t="s">
+        <v>215</v>
+      </c>
       <c r="B29" s="45" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C29" s="45"/>
       <c r="D29" s="24"/>
       <c r="E29" s="46"/>
     </row>
-    <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="25"/>
+    <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="47" t="s">
+        <v>217</v>
+      </c>
       <c r="B30" s="45" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="C30" s="45"/>
       <c r="D30" s="24"/>
       <c r="E30" s="46"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="47" t="s">
-        <v>218</v>
-      </c>
-      <c r="B34" s="45" t="s">
+    <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="47" t="s">
         <v>219</v>
       </c>
-      <c r="C34" s="45"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="46"/>
-    </row>
-    <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="47" t="s">
-        <v>218</v>
-      </c>
-      <c r="B35" s="45" t="s">
+      <c r="B31" s="45" t="s">
         <v>220</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="46"/>
-    </row>
-    <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="47" t="s">
+      <c r="C31" s="45"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="46"/>
+    </row>
+    <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="47" t="s">
         <v>221</v>
       </c>
-      <c r="B36" s="45" t="s">
+      <c r="B32" s="45" t="s">
         <v>222</v>
       </c>
-      <c r="C36" s="45"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="46"/>
-    </row>
-    <row r="37" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="47" t="s">
+      <c r="C32" s="45"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="46"/>
+    </row>
+    <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="47" t="s">
         <v>223</v>
       </c>
-      <c r="B37" s="45" t="s">
+      <c r="B33" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="C37" s="45"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="46"/>
-    </row>
-    <row r="38" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="47" t="s">
+      <c r="C33" s="45"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="46"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="48" t="s">
         <v>225</v>
       </c>
-      <c r="B38" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="C38" s="45"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="46"/>
-    </row>
-    <row r="39" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="47" t="s">
-        <v>227</v>
-      </c>
-      <c r="B39" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="C39" s="45"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="46"/>
-    </row>
-    <row r="40" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="47" t="s">
-        <v>229</v>
-      </c>
-      <c r="B40" s="45" t="s">
-        <v>230</v>
-      </c>
-      <c r="C40" s="45"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="46"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="48" t="s">
-        <v>231</v>
-      </c>
-      <c r="B42" s="48"/>
-      <c r="C42" s="48"/>
-      <c r="D42" s="48"/>
-      <c r="E42" s="48"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="48"/>
-      <c r="B43" s="48"/>
-      <c r="C43" s="48"/>
-      <c r="D43" s="48"/>
-      <c r="E43" s="48"/>
+      <c r="B35" s="48"/>
+      <c r="C35" s="48"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="48"/>
+      <c r="B36" s="48"/>
+      <c r="C36" s="48"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="48"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="28">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A4:E4"/>
@@ -4214,20 +4142,14 @@
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A26:E26"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="A42:E43"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A35:E36"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>